<commit_message>
shrubs and vines updates and cleaned some modelling cures script
</commit_message>
<xml_diff>
--- a/data/MTSV_v2.xlsx
+++ b/data/MTSV_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/christophe_rouleau-desrochers/github/egret/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE3BE6BF-5D28-6847-829B-B07D64C9CFE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{794D65CB-3967-7641-A26A-2946EB3300C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{AB2BA940-7D5B-994D-BF8E-A6F07FAB93DD}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="183">
   <si>
     <t>Family</t>
   </si>
@@ -351,16 +351,260 @@
   </si>
   <si>
     <t>thunbergii</t>
+  </si>
+  <si>
+    <t>Bignoniaceae</t>
+  </si>
+  <si>
+    <t>Campsis</t>
+  </si>
+  <si>
+    <t>radicans</t>
+  </si>
+  <si>
+    <t>Cannabaceae</t>
+  </si>
+  <si>
+    <t>Chamaedaphne</t>
+  </si>
+  <si>
+    <t>calyculata</t>
+  </si>
+  <si>
+    <t>Crateagus</t>
+  </si>
+  <si>
+    <t>chrysocarpa</t>
+  </si>
+  <si>
+    <t>macrosperma</t>
+  </si>
+  <si>
+    <t>punctata</t>
+  </si>
+  <si>
+    <t>succulenta</t>
+  </si>
+  <si>
+    <t>Dasiphora</t>
+  </si>
+  <si>
+    <t>fruticosa</t>
+  </si>
+  <si>
+    <t>fruit persistent through winter</t>
+  </si>
+  <si>
+    <t>Diervillaceae</t>
+  </si>
+  <si>
+    <t>Diervilla</t>
+  </si>
+  <si>
+    <t>lonicera</t>
+  </si>
+  <si>
+    <t>Thymelaeaceae</t>
+  </si>
+  <si>
+    <t>Dirca</t>
+  </si>
+  <si>
+    <t>palustris</t>
+  </si>
+  <si>
+    <t>Epigaea</t>
+  </si>
+  <si>
+    <t>repens</t>
+  </si>
+  <si>
+    <t>Celastraceae</t>
+  </si>
+  <si>
+    <t>Euonymus</t>
+  </si>
+  <si>
+    <t>atropurpureus</t>
+  </si>
+  <si>
+    <t>obovatus</t>
+  </si>
+  <si>
+    <t>Gaultheria</t>
+  </si>
+  <si>
+    <t>hispidula</t>
+  </si>
+  <si>
+    <t>procumbens</t>
+  </si>
+  <si>
+    <t>Hamamelidaceae</t>
+  </si>
+  <si>
+    <t>Hamamelis</t>
+  </si>
+  <si>
+    <t>Hypericaceae</t>
+  </si>
+  <si>
+    <t>Hypericum</t>
+  </si>
+  <si>
+    <t>kalmianum</t>
+  </si>
+  <si>
+    <t>Aquifoliaceae</t>
+  </si>
+  <si>
+    <t>Ilex</t>
+  </si>
+  <si>
+    <t>mucronata</t>
+  </si>
+  <si>
+    <t>communis</t>
+  </si>
+  <si>
+    <t>horizontalis</t>
+  </si>
+  <si>
+    <t>Kalmia</t>
+  </si>
+  <si>
+    <t>angustifolia</t>
+  </si>
+  <si>
+    <t>polifolia</t>
+  </si>
+  <si>
+    <t>Caprifoliaceae</t>
+  </si>
+  <si>
+    <t>Lonicera</t>
+  </si>
+  <si>
+    <t>dioica</t>
+  </si>
+  <si>
+    <t>Menispermaceae</t>
+  </si>
+  <si>
+    <t>Menispermum</t>
+  </si>
+  <si>
+    <t>canadense</t>
+  </si>
+  <si>
+    <t>Vitaceae</t>
+  </si>
+  <si>
+    <t>Parthenocissus</t>
+  </si>
+  <si>
+    <t>inserta</t>
+  </si>
+  <si>
+    <t>Physocarpus</t>
+  </si>
+  <si>
+    <t>opulifolius</t>
+  </si>
+  <si>
+    <t>Rhododendron</t>
+  </si>
+  <si>
+    <t>groenlandicum</t>
+  </si>
+  <si>
+    <t>aromatica</t>
+  </si>
+  <si>
+    <t>copallina</t>
+  </si>
+  <si>
+    <t>Grossulariaceae</t>
+  </si>
+  <si>
+    <t>Ribes</t>
+  </si>
+  <si>
+    <t>cynosbati</t>
+  </si>
+  <si>
+    <t>Rosa</t>
+  </si>
+  <si>
+    <t>blanda</t>
+  </si>
+  <si>
+    <t>multiflora</t>
+  </si>
+  <si>
+    <t>cordata</t>
+  </si>
+  <si>
+    <t>pro/syn</t>
+  </si>
+  <si>
+    <t>myricoides</t>
+  </si>
+  <si>
+    <t>pedicellaris</t>
+  </si>
+  <si>
+    <t>petiolaris</t>
+  </si>
+  <si>
+    <t>serissima</t>
+  </si>
+  <si>
+    <t>Smilacaceae</t>
+  </si>
+  <si>
+    <t>Smilax</t>
+  </si>
+  <si>
+    <t>rotundifolia</t>
+  </si>
+  <si>
+    <t>Solanaceae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solanum </t>
+  </si>
+  <si>
+    <t>dulcamara</t>
+  </si>
+  <si>
+    <t>decora</t>
+  </si>
+  <si>
+    <t>Staphyleaceae</t>
+  </si>
+  <si>
+    <t>Staphylea</t>
+  </si>
+  <si>
+    <t>trifolia</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -386,8 +630,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -722,7 +967,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F4FCE54-EA71-1745-B10B-78ADB8176A52}">
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:J85"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
@@ -1413,7 +1658,7 @@
         <v>89</v>
       </c>
       <c r="B26" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C26" t="s">
         <v>58</v>
@@ -1770,6 +2015,1067 @@
       </c>
       <c r="J39" t="s">
         <v>35</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B40" t="s">
+        <v>104</v>
+      </c>
+      <c r="C40" t="s">
+        <v>105</v>
+      </c>
+      <c r="D40" t="s">
+        <v>106</v>
+      </c>
+      <c r="E40" t="s">
+        <v>75</v>
+      </c>
+      <c r="F40" t="s">
+        <v>14</v>
+      </c>
+      <c r="G40">
+        <v>7.5</v>
+      </c>
+      <c r="H40">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B41" t="s">
+        <v>107</v>
+      </c>
+      <c r="C41" t="s">
+        <v>59</v>
+      </c>
+      <c r="D41" t="s">
+        <v>60</v>
+      </c>
+      <c r="E41" t="s">
+        <v>11</v>
+      </c>
+      <c r="F41" t="s">
+        <v>48</v>
+      </c>
+      <c r="G41">
+        <v>5</v>
+      </c>
+      <c r="H41">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B42" t="s">
+        <v>93</v>
+      </c>
+      <c r="C42" t="s">
+        <v>108</v>
+      </c>
+      <c r="D42" t="s">
+        <v>109</v>
+      </c>
+      <c r="E42" t="s">
+        <v>75</v>
+      </c>
+      <c r="F42" t="s">
+        <v>14</v>
+      </c>
+      <c r="G42">
+        <v>5</v>
+      </c>
+      <c r="H42">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B43" t="s">
+        <v>77</v>
+      </c>
+      <c r="C43" t="s">
+        <v>110</v>
+      </c>
+      <c r="D43" t="s">
+        <v>111</v>
+      </c>
+      <c r="E43" t="s">
+        <v>75</v>
+      </c>
+      <c r="F43" t="s">
+        <v>12</v>
+      </c>
+      <c r="G43">
+        <v>5.5</v>
+      </c>
+      <c r="H43">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B44" t="s">
+        <v>77</v>
+      </c>
+      <c r="C44" t="s">
+        <v>110</v>
+      </c>
+      <c r="D44" t="s">
+        <v>112</v>
+      </c>
+      <c r="E44" t="s">
+        <v>75</v>
+      </c>
+      <c r="F44" t="s">
+        <v>12</v>
+      </c>
+      <c r="G44">
+        <v>5.5</v>
+      </c>
+      <c r="H44">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B45" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C45" t="s">
+        <v>110</v>
+      </c>
+      <c r="D45" t="s">
+        <v>113</v>
+      </c>
+      <c r="E45" t="s">
+        <v>75</v>
+      </c>
+      <c r="F45" t="s">
+        <v>12</v>
+      </c>
+      <c r="G45">
+        <v>5.5</v>
+      </c>
+      <c r="H45">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B46" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C46" t="s">
+        <v>110</v>
+      </c>
+      <c r="D46" t="s">
+        <v>114</v>
+      </c>
+      <c r="E46" t="s">
+        <v>75</v>
+      </c>
+      <c r="F46" t="s">
+        <v>12</v>
+      </c>
+      <c r="G46">
+        <v>5.5</v>
+      </c>
+      <c r="H46">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B47" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C47" t="s">
+        <v>115</v>
+      </c>
+      <c r="D47" t="s">
+        <v>116</v>
+      </c>
+      <c r="E47" t="s">
+        <v>75</v>
+      </c>
+      <c r="F47" t="s">
+        <v>14</v>
+      </c>
+      <c r="G47">
+        <v>7.5</v>
+      </c>
+      <c r="H47" t="s">
+        <v>14</v>
+      </c>
+      <c r="J47" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B48" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="C48" t="s">
+        <v>119</v>
+      </c>
+      <c r="D48" t="s">
+        <v>120</v>
+      </c>
+      <c r="E48" t="s">
+        <v>75</v>
+      </c>
+      <c r="F48" t="s">
+        <v>14</v>
+      </c>
+      <c r="G48">
+        <v>6</v>
+      </c>
+      <c r="H48">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="49" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B49" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C49" t="s">
+        <v>122</v>
+      </c>
+      <c r="D49" t="s">
+        <v>123</v>
+      </c>
+      <c r="E49" t="s">
+        <v>75</v>
+      </c>
+      <c r="F49" t="s">
+        <v>48</v>
+      </c>
+      <c r="G49">
+        <v>4.5</v>
+      </c>
+      <c r="H49">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="50" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B50" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C50" t="s">
+        <v>124</v>
+      </c>
+      <c r="D50" t="s">
+        <v>125</v>
+      </c>
+      <c r="E50" t="s">
+        <v>75</v>
+      </c>
+      <c r="F50" t="s">
+        <v>14</v>
+      </c>
+      <c r="G50">
+        <v>4.5</v>
+      </c>
+      <c r="H50" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="51" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B51" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C51" t="s">
+        <v>127</v>
+      </c>
+      <c r="D51" t="s">
+        <v>128</v>
+      </c>
+      <c r="E51" t="s">
+        <v>75</v>
+      </c>
+      <c r="F51" t="s">
+        <v>14</v>
+      </c>
+      <c r="G51">
+        <v>6</v>
+      </c>
+      <c r="H51">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B52" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C52" t="s">
+        <v>127</v>
+      </c>
+      <c r="D52" t="s">
+        <v>129</v>
+      </c>
+      <c r="E52" t="s">
+        <v>75</v>
+      </c>
+      <c r="F52" t="s">
+        <v>14</v>
+      </c>
+      <c r="G52">
+        <v>4.5</v>
+      </c>
+      <c r="H52">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B53" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C53" t="s">
+        <v>130</v>
+      </c>
+      <c r="D53" t="s">
+        <v>131</v>
+      </c>
+      <c r="E53" t="s">
+        <v>75</v>
+      </c>
+      <c r="F53" t="s">
+        <v>14</v>
+      </c>
+      <c r="G53">
+        <v>5.5</v>
+      </c>
+      <c r="H53">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="54" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B54" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C54" t="s">
+        <v>130</v>
+      </c>
+      <c r="D54" t="s">
+        <v>132</v>
+      </c>
+      <c r="E54" t="s">
+        <v>75</v>
+      </c>
+      <c r="F54" t="s">
+        <v>14</v>
+      </c>
+      <c r="G54">
+        <v>7.5</v>
+      </c>
+      <c r="H54">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="55" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B55" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C55" t="s">
+        <v>134</v>
+      </c>
+      <c r="D55" t="s">
+        <v>41</v>
+      </c>
+      <c r="E55" t="s">
+        <v>75</v>
+      </c>
+      <c r="F55" t="s">
+        <v>76</v>
+      </c>
+      <c r="G55">
+        <v>10.5</v>
+      </c>
+      <c r="H55" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="56" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B56" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C56" t="s">
+        <v>136</v>
+      </c>
+      <c r="D56" t="s">
+        <v>137</v>
+      </c>
+      <c r="E56" t="s">
+        <v>75</v>
+      </c>
+      <c r="F56" t="s">
+        <v>14</v>
+      </c>
+      <c r="G56">
+        <v>7.5</v>
+      </c>
+      <c r="H56">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="57" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B57" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C57" t="s">
+        <v>139</v>
+      </c>
+      <c r="D57" t="s">
+        <v>140</v>
+      </c>
+      <c r="E57" t="s">
+        <v>75</v>
+      </c>
+      <c r="F57" t="s">
+        <v>48</v>
+      </c>
+      <c r="G57">
+        <v>5</v>
+      </c>
+      <c r="H57">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="58" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B58" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C58" t="s">
+        <v>40</v>
+      </c>
+      <c r="D58" t="s">
+        <v>141</v>
+      </c>
+      <c r="E58" t="s">
+        <v>11</v>
+      </c>
+      <c r="F58" t="s">
+        <v>14</v>
+      </c>
+      <c r="G58">
+        <v>5.5</v>
+      </c>
+      <c r="H58" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="59" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B59" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C59" t="s">
+        <v>40</v>
+      </c>
+      <c r="D59" t="s">
+        <v>142</v>
+      </c>
+      <c r="E59" t="s">
+        <v>11</v>
+      </c>
+      <c r="F59" t="s">
+        <v>14</v>
+      </c>
+      <c r="G59" t="s">
+        <v>14</v>
+      </c>
+      <c r="H59" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="60" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B60" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C60" t="s">
+        <v>143</v>
+      </c>
+      <c r="D60" t="s">
+        <v>144</v>
+      </c>
+      <c r="E60" t="s">
+        <v>75</v>
+      </c>
+      <c r="F60" t="s">
+        <v>14</v>
+      </c>
+      <c r="G60">
+        <v>6.5</v>
+      </c>
+      <c r="H60" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="61" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B61" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C61" t="s">
+        <v>143</v>
+      </c>
+      <c r="D61" t="s">
+        <v>145</v>
+      </c>
+      <c r="E61" t="s">
+        <v>75</v>
+      </c>
+      <c r="F61" t="s">
+        <v>14</v>
+      </c>
+      <c r="G61">
+        <v>5.5</v>
+      </c>
+      <c r="H61" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="62" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B62" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C62" t="s">
+        <v>147</v>
+      </c>
+      <c r="D62" t="s">
+        <v>39</v>
+      </c>
+      <c r="E62" t="s">
+        <v>75</v>
+      </c>
+      <c r="F62" t="s">
+        <v>14</v>
+      </c>
+      <c r="G62">
+        <v>5.5</v>
+      </c>
+      <c r="H62">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="63" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B63" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C63" t="s">
+        <v>147</v>
+      </c>
+      <c r="D63" t="s">
+        <v>148</v>
+      </c>
+      <c r="E63" t="s">
+        <v>75</v>
+      </c>
+      <c r="F63" t="s">
+        <v>14</v>
+      </c>
+      <c r="G63">
+        <v>5.5</v>
+      </c>
+      <c r="H63">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="64" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B64" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="C64" t="s">
+        <v>150</v>
+      </c>
+      <c r="D64" t="s">
+        <v>151</v>
+      </c>
+      <c r="E64" t="s">
+        <v>75</v>
+      </c>
+      <c r="F64" t="s">
+        <v>14</v>
+      </c>
+      <c r="G64">
+        <v>6</v>
+      </c>
+      <c r="H64">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="65" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B65" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C65" t="s">
+        <v>153</v>
+      </c>
+      <c r="D65" t="s">
+        <v>154</v>
+      </c>
+      <c r="E65" t="s">
+        <v>75</v>
+      </c>
+      <c r="F65" t="s">
+        <v>14</v>
+      </c>
+      <c r="G65">
+        <v>6.5</v>
+      </c>
+      <c r="H65">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="66" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B66" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C66" t="s">
+        <v>155</v>
+      </c>
+      <c r="D66" t="s">
+        <v>156</v>
+      </c>
+      <c r="E66" t="s">
+        <v>75</v>
+      </c>
+      <c r="F66" t="s">
+        <v>14</v>
+      </c>
+      <c r="G66">
+        <v>5.5</v>
+      </c>
+      <c r="H66">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="67" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B67" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C67" t="s">
+        <v>61</v>
+      </c>
+      <c r="D67" t="s">
+        <v>62</v>
+      </c>
+      <c r="E67" t="s">
+        <v>11</v>
+      </c>
+      <c r="F67" t="s">
+        <v>12</v>
+      </c>
+      <c r="G67">
+        <v>5</v>
+      </c>
+      <c r="H67" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="68" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B68" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C68" t="s">
+        <v>157</v>
+      </c>
+      <c r="D68" t="s">
+        <v>158</v>
+      </c>
+      <c r="E68" t="s">
+        <v>75</v>
+      </c>
+      <c r="F68" t="s">
+        <v>14</v>
+      </c>
+      <c r="G68">
+        <v>5.5</v>
+      </c>
+      <c r="H68">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="69" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B69" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D69" t="s">
+        <v>159</v>
+      </c>
+      <c r="E69" t="s">
+        <v>75</v>
+      </c>
+      <c r="F69" t="s">
+        <v>48</v>
+      </c>
+      <c r="G69">
+        <v>4.5</v>
+      </c>
+      <c r="H69">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="70" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B70" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D70" t="s">
+        <v>160</v>
+      </c>
+      <c r="E70" t="s">
+        <v>75</v>
+      </c>
+      <c r="F70" t="s">
+        <v>14</v>
+      </c>
+      <c r="G70">
+        <v>6.5</v>
+      </c>
+      <c r="H70">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B71" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D71" t="s">
+        <v>67</v>
+      </c>
+      <c r="E71" t="s">
+        <v>75</v>
+      </c>
+      <c r="F71" t="s">
+        <v>76</v>
+      </c>
+      <c r="G71">
+        <v>6</v>
+      </c>
+      <c r="H71">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="72" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B72" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="D72" t="s">
+        <v>163</v>
+      </c>
+      <c r="E72" t="s">
+        <v>75</v>
+      </c>
+      <c r="F72" t="s">
+        <v>14</v>
+      </c>
+      <c r="G72">
+        <v>4.5</v>
+      </c>
+      <c r="H72">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="73" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B73" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="D73" t="s">
+        <v>165</v>
+      </c>
+      <c r="E73" t="s">
+        <v>75</v>
+      </c>
+      <c r="F73" t="s">
+        <v>14</v>
+      </c>
+      <c r="G73">
+        <v>5.5</v>
+      </c>
+      <c r="H73">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B74" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="D74" t="s">
+        <v>166</v>
+      </c>
+      <c r="E74" t="s">
+        <v>75</v>
+      </c>
+      <c r="F74" t="s">
+        <v>14</v>
+      </c>
+      <c r="G74">
+        <v>5.5</v>
+      </c>
+      <c r="H74">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="75" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B75" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D75" t="s">
+        <v>167</v>
+      </c>
+      <c r="E75" t="s">
+        <v>74</v>
+      </c>
+      <c r="F75" t="s">
+        <v>168</v>
+      </c>
+      <c r="G75">
+        <v>5.5</v>
+      </c>
+      <c r="H75">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="76" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B76" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D76" t="s">
+        <v>169</v>
+      </c>
+      <c r="E76" t="s">
+        <v>74</v>
+      </c>
+      <c r="F76" t="s">
+        <v>168</v>
+      </c>
+      <c r="G76">
+        <v>5.5</v>
+      </c>
+      <c r="H76">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="77" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B77" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D77" t="s">
+        <v>170</v>
+      </c>
+      <c r="E77" t="s">
+        <v>74</v>
+      </c>
+      <c r="F77" t="s">
+        <v>12</v>
+      </c>
+      <c r="G77">
+        <v>5.5</v>
+      </c>
+      <c r="H77">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="78" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B78" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D78" t="s">
+        <v>171</v>
+      </c>
+      <c r="E78" t="s">
+        <v>74</v>
+      </c>
+      <c r="F78" t="s">
+        <v>12</v>
+      </c>
+      <c r="G78">
+        <v>5.5</v>
+      </c>
+      <c r="H78">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="79" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B79" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D79" t="s">
+        <v>172</v>
+      </c>
+      <c r="E79" t="s">
+        <v>74</v>
+      </c>
+      <c r="F79" t="s">
+        <v>76</v>
+      </c>
+      <c r="G79">
+        <v>5.5</v>
+      </c>
+      <c r="H79">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B80" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="D80" t="s">
+        <v>94</v>
+      </c>
+      <c r="E80" t="s">
+        <v>75</v>
+      </c>
+      <c r="F80" t="s">
+        <v>14</v>
+      </c>
+      <c r="G80">
+        <v>6</v>
+      </c>
+      <c r="H80">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="81" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B81" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="D81" t="s">
+        <v>175</v>
+      </c>
+      <c r="E81" t="s">
+        <v>75</v>
+      </c>
+      <c r="F81" t="s">
+        <v>14</v>
+      </c>
+      <c r="G81">
+        <v>6</v>
+      </c>
+      <c r="H81">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="82" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B82" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="D82" t="s">
+        <v>178</v>
+      </c>
+      <c r="E82" t="s">
+        <v>75</v>
+      </c>
+      <c r="F82" t="s">
+        <v>14</v>
+      </c>
+      <c r="G82">
+        <v>7</v>
+      </c>
+      <c r="H82">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B83" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D83" t="s">
+        <v>56</v>
+      </c>
+      <c r="E83" t="s">
+        <v>75</v>
+      </c>
+      <c r="F83" t="s">
+        <v>76</v>
+      </c>
+      <c r="G83">
+        <v>5.5</v>
+      </c>
+      <c r="H83">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="84" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B84" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D84" t="s">
+        <v>179</v>
+      </c>
+      <c r="E84" t="s">
+        <v>75</v>
+      </c>
+      <c r="F84" t="s">
+        <v>76</v>
+      </c>
+      <c r="G84">
+        <v>6.5</v>
+      </c>
+      <c r="H84">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="85" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B85" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="D85" t="s">
+        <v>182</v>
+      </c>
+      <c r="E85" t="s">
+        <v>75</v>
+      </c>
+      <c r="F85" t="s">
+        <v>168</v>
+      </c>
+      <c r="G85">
+        <v>4.5</v>
+      </c>
+      <c r="H85">
+        <v>9.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>